<commit_message>
breakdown edits, other edits
</commit_message>
<xml_diff>
--- a/results/03-2026/beta/contributions-03-2026.xlsx
+++ b/results/03-2026/beta/contributions-03-2026.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -105,6 +105,12 @@
   </si>
   <si>
     <t xml:space="preserve">fiscal_impact_4q_ma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">taxes_breakdown_contribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transfers_breakdown_contribution</t>
   </si>
   <si>
     <t xml:space="preserve">2020 Q1</t>
@@ -629,13 +635,19 @@
       <c r="AE1" t="s">
         <v>30</v>
       </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -723,14 +735,20 @@
       </c>
       <c r="AE2" t="n">
         <v>0.577601160588483</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>-0.0917203334476128</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0.133565386955577</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
@@ -818,14 +836,20 @@
       </c>
       <c r="AE3" t="n">
         <v>3.00961320689186</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0.218260041490563</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>8.62039918521447</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
         <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>32</v>
       </c>
       <c r="C4" t="n">
         <v>-1</v>
@@ -913,14 +937,20 @@
       </c>
       <c r="AE4" t="n">
         <v>3.83799587371516</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0.552346472186169</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>4.96184053113914</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="n">
         <v>-1</v>
@@ -1008,14 +1038,20 @@
       </c>
       <c r="AE5" t="n">
         <v>2.90763406238303</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>-0.568772712361355</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>-2.48939682148616</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" t="n">
         <v>-1</v>
@@ -1103,14 +1139,20 @@
       </c>
       <c r="AE6" t="n">
         <v>4.92390395761885</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>-0.193345941150108</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>7.80632121184456</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C7" t="n">
         <v>-1</v>
@@ -1198,14 +1240,20 @@
       </c>
       <c r="AE7" t="n">
         <v>1.71389535669892</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>-0.24689103402653</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>-1.07983609284451</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" t="n">
         <v>-1</v>
@@ -1293,14 +1341,20 @@
       </c>
       <c r="AE8" t="n">
         <v>-0.106007963281536</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>-0.31515314337929</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>-2.09021198351942</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C9" t="n">
         <v>-1</v>
@@ -1388,14 +1442,20 @@
       </c>
       <c r="AE9" t="n">
         <v>-0.0643244424293917</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>-0.208789857580898</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>-2.44671974554818</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C10" t="n">
         <v>-1</v>
@@ -1483,14 +1543,20 @@
       </c>
       <c r="AE10" t="n">
         <v>-3.19423837869211</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>-0.876075859460641</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>-2.18229105712882</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C11" t="n">
         <v>-1</v>
@@ -1578,14 +1644,20 @@
       </c>
       <c r="AE11" t="n">
         <v>-3.83451695668526</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>-1.20568398792863</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>-3.10254365284433</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C12" t="n">
         <v>-1</v>
@@ -1673,14 +1745,20 @@
       </c>
       <c r="AE12" t="n">
         <v>-3.62581383024339</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>-0.657494577538429</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>-1.71450742085577</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" t="n">
         <v>-1</v>
@@ -1768,14 +1846,20 @@
       </c>
       <c r="AE13" t="n">
         <v>-2.98274687443948</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>-0.332348599335242</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>-0.443743756909895</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C14" t="n">
         <v>-1</v>
@@ -1863,14 +1947,20 @@
       </c>
       <c r="AE14" t="n">
         <v>-2.02726920885071</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>0.46615754920793</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>-1.24231811101493</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C15" t="n">
         <v>-1</v>
@@ -1958,14 +2048,20 @@
       </c>
       <c r="AE15" t="n">
         <v>-0.89685239280325</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0.528053936044742</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>-1.38247728801657</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C16" t="n">
         <v>-1</v>
@@ -2053,14 +2149,20 @@
       </c>
       <c r="AE16" t="n">
         <v>-0.271579396961083</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0.18171700258577</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>-0.657570272399199</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C17" t="n">
         <v>-1</v>
@@ -2148,14 +2250,20 @@
       </c>
       <c r="AE17" t="n">
         <v>-0.223361959702328</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>0.0862390375637294</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>-0.663214681106842</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C18" t="n">
         <v>-1</v>
@@ -2243,14 +2351,20 @@
       </c>
       <c r="AE18" t="n">
         <v>-0.140039015352823</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>0.659854636965577</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>-0.455077977525216</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C19" t="n">
         <v>-1</v>
@@ -2338,14 +2452,20 @@
       </c>
       <c r="AE19" t="n">
         <v>0.048470906359604</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0.508714905565415</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>-0.384591213069866</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C20" t="n">
         <v>-1</v>
@@ -2402,7 +2522,7 @@
         <v>-0.0440281009267043</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.055339761076515</v>
+        <v>-0.0553398426809612</v>
       </c>
       <c r="V20" t="n">
         <v>-0.0000481981319541984</v>
@@ -2423,24 +2543,30 @@
         <v>0.180384979214747</v>
       </c>
       <c r="AB20" t="n">
-        <v>-0.0742381544293124</v>
+        <v>-0.0742382360498926</v>
       </c>
       <c r="AC20" t="n">
-        <v>0.106287009376921</v>
+        <v>0.106286927910456</v>
       </c>
       <c r="AD20" t="n">
-        <v>0.601612110807237</v>
+        <v>0.601612029340773</v>
       </c>
       <c r="AE20" t="n">
-        <v>0.186985184633372</v>
+        <v>0.186985164266756</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>0.274816107829201</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>-0.0188983933689314</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C21" t="n">
         <v>-1</v>
@@ -2497,7 +2623,7 @@
         <v>-0.0265684363093117</v>
       </c>
       <c r="U21" t="n">
-        <v>-0.0302912960815929</v>
+        <v>-0.0302912288977294</v>
       </c>
       <c r="V21" t="n">
         <v>-0.0000584549268793934</v>
@@ -2518,24 +2644,30 @@
         <v>0.168699850674615</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.203974267353671</v>
+        <v>0.203974334374208</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.372316942334643</v>
+        <v>0.37231700923784</v>
       </c>
       <c r="AD21" t="n">
-        <v>0.511324389373289</v>
+        <v>0.511324456276486</v>
       </c>
       <c r="AE21" t="n">
-        <v>0.382038254203639</v>
+        <v>0.382038250562822</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>0.303037201695179</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>0.234265563271938</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C22" t="n">
         <v>-1</v>
@@ -2592,7 +2724,7 @@
         <v>-0.0106418570513199</v>
       </c>
       <c r="U22" t="n">
-        <v>-0.0297652464367883</v>
+        <v>-0.0297652241785434</v>
       </c>
       <c r="V22" t="n">
         <v>-0.000305138334205149</v>
@@ -2613,24 +2745,30 @@
         <v>-0.0973949910447126</v>
       </c>
       <c r="AB22" t="n">
-        <v>-0.00437634796183327</v>
+        <v>-0.00437632570967921</v>
       </c>
       <c r="AC22" t="n">
-        <v>-0.101775840139854</v>
+        <v>-0.101775817864685</v>
       </c>
       <c r="AD22" t="n">
-        <v>-0.695053695338983</v>
+        <v>-0.695053673063814</v>
       </c>
       <c r="AE22" t="n">
-        <v>0.165772303006992</v>
+        <v>0.165772304934967</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>0.0179122702725422</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>0.0253888984688642</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C23" t="n">
         <v>-1</v>
@@ -2687,7 +2825,7 @@
         <v>-0.0100206453912311</v>
       </c>
       <c r="U23" t="n">
-        <v>-0.0233355697699924</v>
+        <v>-0.0233356501478242</v>
       </c>
       <c r="V23" t="n">
         <v>-0.00103802633880351</v>
@@ -2708,24 +2846,30 @@
         <v>-0.274529505412121</v>
       </c>
       <c r="AB23" t="n">
-        <v>0.445899459268899</v>
+        <v>0.445899379286268</v>
       </c>
       <c r="AC23" t="n">
-        <v>-0.0273474449240554</v>
+        <v>-0.0273475251368821</v>
       </c>
       <c r="AD23" t="n">
-        <v>-0.433189323644773</v>
+        <v>-0.4331894038576</v>
       </c>
       <c r="AE23" t="n">
-        <v>-0.00382662970080774</v>
+        <v>-0.00382664782603897</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>-0.491452879857937</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0.469235029434092</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C24" t="n">
         <v>-1</v>
@@ -2782,7 +2926,7 @@
         <v>-0.0086306387520275</v>
       </c>
       <c r="U24" t="n">
-        <v>-0.0297886168486114</v>
+        <v>-0.0297549970186519</v>
       </c>
       <c r="V24" t="n">
         <v>-0.0000539507371187338</v>
@@ -2803,24 +2947,30 @@
         <v>-0.139229581720164</v>
       </c>
       <c r="AB24" t="n">
-        <v>0.400799604954009</v>
+        <v>0.400833075000047</v>
       </c>
       <c r="AC24" t="n">
-        <v>0.262147478565033</v>
+        <v>0.262180996866793</v>
       </c>
       <c r="AD24" t="n">
-        <v>0.260281409061421</v>
+        <v>0.26031492736318</v>
       </c>
       <c r="AE24" t="n">
-        <v>-0.0891593051372617</v>
+        <v>-0.089150923320437</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>-0.373161504158873</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0.430588072018699</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C25" t="n">
         <v>-1</v>
@@ -2877,7 +3027,7 @@
         <v>-0.00768147033983896</v>
       </c>
       <c r="U25" t="n">
-        <v>-0.0243002856780776</v>
+        <v>-0.0243055898647292</v>
       </c>
       <c r="V25" t="n">
         <v>-0.000053641022635247</v>
@@ -2898,24 +3048,30 @@
         <v>-0.246604197090628</v>
       </c>
       <c r="AB25" t="n">
-        <v>0.359395773669213</v>
+        <v>0.359390490912369</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.113724678699862</v>
+        <v>0.113719382218795</v>
       </c>
       <c r="AD25" t="n">
-        <v>-1.23625881023253</v>
+        <v>-1.2362641067136</v>
       </c>
       <c r="AE25" t="n">
-        <v>-0.526055105038717</v>
+        <v>-0.526048064067958</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>-0.389037106947415</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>0.383696080777098</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C26" t="n">
         <v>0</v>
@@ -2924,7 +3080,7 @@
         <v>1.66203965967879</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.188444884734299</v>
+        <v>-10.958502461799</v>
       </c>
       <c r="F26" t="n">
         <v>-0.0884930148988476</v>
@@ -2972,7 +3128,7 @@
         <v>-0.00705294137280971</v>
       </c>
       <c r="U26" t="n">
-        <v>-0.0223732761489481</v>
+        <v>-0.0223752480478402</v>
       </c>
       <c r="V26" t="n">
         <v>-0.000508719097945849</v>
@@ -2984,33 +3140,39 @@
         <v>0.0459340379109913</v>
       </c>
       <c r="Y26" t="n">
-        <v>1.61105778904093</v>
+        <v>0.0781758139260642</v>
       </c>
       <c r="Z26" t="n">
-        <v>-0.137463014096444</v>
+        <v>-9.37463861604627</v>
       </c>
       <c r="AA26" t="n">
         <v>0.258500252640078</v>
       </c>
       <c r="AB26" t="n">
-        <v>0.334539830180878</v>
+        <v>0.334537865725155</v>
       </c>
       <c r="AC26" t="n">
-        <v>0.652124840640011</v>
+        <v>0.65212288156191</v>
       </c>
       <c r="AD26" t="n">
-        <v>2.1257196155845</v>
+        <v>-8.6443399205583</v>
       </c>
       <c r="AE26" t="n">
-        <v>0.179138222692154</v>
+        <v>-2.51336962594158</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>-0.0572575248558411</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0.356913113772995</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B27" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -3019,7 +3181,7 @@
         <v>-0.420442225197428</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.175941628331148</v>
+        <v>-0.0000851769538371798</v>
       </c>
       <c r="F27" t="n">
         <v>-0.0484841727550417</v>
@@ -3067,7 +3229,7 @@
         <v>-0.00646180404202451</v>
       </c>
       <c r="U27" t="n">
-        <v>-0.0205148231023012</v>
+        <v>-0.0205167048643551</v>
       </c>
       <c r="V27" t="n">
         <v>-0.000434592407571766</v>
@@ -3079,33 +3241,39 @@
         <v>0.0500663295646562</v>
       </c>
       <c r="Y27" t="n">
-        <v>-0.504761266635606</v>
+        <v>-0.503775436537204</v>
       </c>
       <c r="Z27" t="n">
-        <v>-0.09162258689297</v>
+        <v>0.0832480343859387</v>
       </c>
       <c r="AA27" t="n">
         <v>0.231146628054871</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.102373415401532</v>
+        <v>0.102371536071816</v>
       </c>
       <c r="AC27" t="n">
-        <v>0.39327098033247</v>
+        <v>0.393269105575715</v>
       </c>
       <c r="AD27" t="n">
-        <v>-0.203112873196107</v>
+        <v>-0.0272582965755501</v>
       </c>
       <c r="AE27" t="n">
-        <v>0.23665733530432</v>
+        <v>-2.41188684912107</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>-0.0205269321072229</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0.122888240936171</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" t="s">
         <v>59</v>
-      </c>
-      <c r="B28" t="s">
-        <v>57</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -3114,7 +3282,7 @@
         <v>-0.150762188480544</v>
       </c>
       <c r="E28" t="n">
-        <v>-0.174802504544369</v>
+        <v>-0.000084879505190921</v>
       </c>
       <c r="F28" t="n">
         <v>-0.105484963636033</v>
@@ -3162,7 +3330,7 @@
         <v>-0.00574407026248544</v>
       </c>
       <c r="U28" t="n">
-        <v>-0.0194249836830286</v>
+        <v>-0.0194346552529259</v>
       </c>
       <c r="V28" t="n">
         <v>-0.000402363632723511</v>
@@ -3174,33 +3342,39 @@
         <v>-0.00902525902619576</v>
       </c>
       <c r="Y28" t="n">
-        <v>-0.18691079692726</v>
+        <v>-0.186873183932222</v>
       </c>
       <c r="Z28" t="n">
-        <v>-0.138653896097653</v>
+        <v>0.0360261159464873</v>
       </c>
       <c r="AA28" t="n">
         <v>0.00571655826186169</v>
       </c>
       <c r="AB28" t="n">
-        <v>0.19452277010418</v>
+        <v>0.194513120390624</v>
       </c>
       <c r="AC28" t="n">
-        <v>0.260227579794373</v>
+        <v>0.260217930663832</v>
       </c>
       <c r="AD28" t="n">
-        <v>-0.0653371132305395</v>
+        <v>0.109370862678097</v>
       </c>
       <c r="AE28" t="n">
-        <v>0.15525270473133</v>
+        <v>-2.44962286529234</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>-0.0722545818014097</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>0.21394777564355</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
@@ -3209,7 +3383,7 @@
         <v>-0.110103309128598</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.198319979800335</v>
+        <v>-0.00137907822692901</v>
       </c>
       <c r="F29" t="n">
         <v>-0.0898711501606448</v>
@@ -3257,7 +3431,7 @@
         <v>-0.00316614462247006</v>
       </c>
       <c r="U29" t="n">
-        <v>-0.0123084447393558</v>
+        <v>-0.0123148070021903</v>
       </c>
       <c r="V29" t="n">
         <v>-0.000371323587931648</v>
@@ -3269,33 +3443,39 @@
         <v>-0.0362315364137063</v>
       </c>
       <c r="Y29" t="n">
-        <v>-0.169025391480398</v>
+        <v>-0.167623995548349</v>
       </c>
       <c r="Z29" t="n">
-        <v>-0.139397897448535</v>
+        <v>0.056141608192822</v>
       </c>
       <c r="AA29" t="n">
         <v>-0.107053821905824</v>
       </c>
       <c r="AB29" t="n">
-        <v>0.179109120512849</v>
+        <v>0.179102771157839</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.132258518226359</v>
+        <v>0.132252161664947</v>
       </c>
       <c r="AD29" t="n">
-        <v>-0.176164770702574</v>
+        <v>0.02076977430942</v>
       </c>
       <c r="AE29" t="n">
-        <v>0.420276214613819</v>
+        <v>-2.13536439503658</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>-0.0547348704487144</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>0.191417578160029</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B30" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
@@ -3304,7 +3484,7 @@
         <v>-0.117417360335764</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.184699668516127</v>
+        <v>0.00187897068140066</v>
       </c>
       <c r="F30" t="n">
         <v>-0.341926351241659</v>
@@ -3352,7 +3532,7 @@
         <v>-0.00178043780722077</v>
       </c>
       <c r="U30" t="n">
-        <v>-0.0116901087426907</v>
+        <v>-0.0116901955682493</v>
       </c>
       <c r="V30" t="n">
         <v>-0.000322751259010612</v>
@@ -3364,33 +3544,39 @@
         <v>-0.0191721781779693</v>
       </c>
       <c r="Y30" t="n">
-        <v>-0.163489049151569</v>
+        <v>-0.162650305358439</v>
       </c>
       <c r="Z30" t="n">
-        <v>-0.138627979700321</v>
+        <v>0.0471119157040758</v>
       </c>
       <c r="AA30" t="n">
         <v>-0.564485461478001</v>
       </c>
       <c r="AB30" t="n">
-        <v>0.109796463318841</v>
+        <v>0.109796376605536</v>
       </c>
       <c r="AC30" t="n">
-        <v>-0.394030419437947</v>
+        <v>-0.39403050667149</v>
       </c>
       <c r="AD30" t="n">
-        <v>-0.696147448289838</v>
+        <v>-0.509568896325853</v>
       </c>
       <c r="AE30" t="n">
-        <v>-0.285190551354765</v>
+        <v>-0.101671638978471</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>-0.297470801393531</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0.121486572173785</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B31" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
@@ -3399,7 +3585,7 @@
         <v>-0.100473963438391</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.179270880833719</v>
+        <v>0.00163362218100636</v>
       </c>
       <c r="F31" t="n">
         <v>-0.204786789431061</v>
@@ -3447,7 +3633,7 @@
         <v>-0.00149818167456064</v>
       </c>
       <c r="U31" t="n">
-        <v>-0.00977296194688904</v>
+        <v>-0.00977454160018567</v>
       </c>
       <c r="V31" t="n">
         <v>-0.000315399360043053</v>
@@ -3459,33 +3645,39 @@
         <v>-0.0263285513735382</v>
       </c>
       <c r="Y31" t="n">
-        <v>-0.144849501312543</v>
+        <v>-0.144239404558048</v>
       </c>
       <c r="Z31" t="n">
-        <v>-0.134895342959567</v>
+        <v>0.0453990633006634</v>
       </c>
       <c r="AA31" t="n">
         <v>-0.514519464576806</v>
       </c>
       <c r="AB31" t="n">
-        <v>0.0581216072125231</v>
+        <v>0.0581200287022978</v>
       </c>
       <c r="AC31" t="n">
-        <v>-0.396079368670447</v>
+        <v>-0.396080955831403</v>
       </c>
       <c r="AD31" t="n">
-        <v>-0.675824212942557</v>
+        <v>-0.494921297088788</v>
       </c>
       <c r="AE31" t="n">
-        <v>-0.403368386291377</v>
+        <v>-0.21858738910678</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>-0.150504478130735</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>0.0678945703024835</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B32" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -3494,7 +3686,7 @@
         <v>-0.107299968256074</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.18649358757554</v>
+        <v>-0.000933234579202482</v>
       </c>
       <c r="F32" t="n">
         <v>0.034233844104934</v>
@@ -3542,7 +3734,7 @@
         <v>-0.00123825675895601</v>
       </c>
       <c r="U32" t="n">
-        <v>0.0249260452479259</v>
+        <v>0.0249199937637267</v>
       </c>
       <c r="V32" t="n">
         <v>-0.000309166722110859</v>
@@ -3554,33 +3746,39 @@
         <v>-0.0417236588915249</v>
       </c>
       <c r="Y32" t="n">
-        <v>-0.149995756965964</v>
+        <v>-0.14958715383456</v>
       </c>
       <c r="Z32" t="n">
-        <v>-0.14379779886565</v>
+        <v>0.0413539509992837</v>
       </c>
       <c r="AA32" t="n">
         <v>-0.298964935396437</v>
       </c>
       <c r="AB32" t="n">
-        <v>0.0255165371813811</v>
+        <v>0.0255104857351777</v>
       </c>
       <c r="AC32" t="n">
-        <v>-0.273367193246684</v>
+        <v>-0.273373263952081</v>
       </c>
       <c r="AD32" t="n">
-        <v>-0.567160749078297</v>
+        <v>-0.381606466787357</v>
       </c>
       <c r="AE32" t="n">
-        <v>-0.528824295253317</v>
+        <v>-0.341331721473144</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>0.0876690554203386</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>0.000590491971451036</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B33" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C33" t="n">
         <v>0</v>
@@ -3589,7 +3787,7 @@
         <v>-0.177189931468643</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.182994301623059</v>
+        <v>-0.0000601512990431544</v>
       </c>
       <c r="F33" t="n">
         <v>0.0724754946545994</v>
@@ -3649,10 +3847,10 @@
         <v>-0.0185165001078903</v>
       </c>
       <c r="Y33" t="n">
-        <v>-0.218468095965497</v>
+        <v>-0.218395145140965</v>
       </c>
       <c r="Z33" t="n">
-        <v>-0.141716137126205</v>
+        <v>0.0411450623732785</v>
       </c>
       <c r="AA33" t="n">
         <v>-0.288652119497053</v>
@@ -3664,10 +3862,16 @@
         <v>-0.287339460246776</v>
       </c>
       <c r="AD33" t="n">
-        <v>-0.647523693338478</v>
+        <v>-0.464589543014462</v>
       </c>
       <c r="AE33" t="n">
-        <v>-0.646664025912293</v>
+        <v>-0.462671550804114</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0.140292342306064</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>-0.0205292912419754</v>
       </c>
     </row>
   </sheetData>

</xml_diff>